<commit_message>
V2: Complete Resume Parser with Advanced NLP and GPT Integration
- Implemented comprehensive field extraction for all required HR fields
- Added advanced NLP processing with spaCy and NLTK
- Integrated OpenAI GPT for field validation and correction
- Enhanced OCR support with better error handling
- Added structured CSV/Excel output with all specified columns
- Improved name extraction from filenames and text
- Added detailed education, projects, certificates parsing
- Implemented skills categorization (core, people, tech)
- Added work experience and activities extraction
- Better error handling and progress reporting
- Support for multiple file formats (PDF, DOCX, images)
- Comprehensive field validation and data cleaning
</commit_message>
<xml_diff>
--- a/resume_analysis.xlsx
+++ b/resume_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,1099 +436,2507 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Courses</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Course Levels</t>
+          <t>Programme</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Certifications</t>
+          <t>Batch</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Probability</t>
+          <t>Major_Specialization</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Minor_Specialization</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Professional_Summary</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>CoCurricular</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ExtraCurricular</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Top_Core_Skills</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Top_People_Skills</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Top_Tech_Skills</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Certificates</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Work_Experience</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NihalPardeshi_ComputerEngineeringAIML - Nihal Pardeshi.pdf</t>
+          <t>MansiBharatEvre_ComputerEngineering - Mansi Evre.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development', 'Cloud Computing']</t>
+          <t>MANSI EVRE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Advanced', 'Web Development': 'Advanced', 'Cloud Computing': 'Advanced'}</t>
+          <t>12th</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>3.4</v>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AI engineering</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>To secure an AI engineering role where I can utilize expertise in machine learning, natural language processing, and neural networks to develop innovative AI solutions, enhance operational efficiency, and drive data-driven decision-making for organizational success.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Dance, Exploring new places</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>HSC - 12th from Sinhgad college of science ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Enhancing security in Sustainable Vending Machines through advanced techniques () -</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Participating in Singapore conference by  (); Nature based solution for disaster and climate resilience by  ()</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VarunInamdar_ArtificialIntelligence - Varun Inamdar.pdf</t>
+          <t>Srushti Jujare-Resume - Srushti Jujare.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development', 'Cloud Computing']</t>
+          <t>SRUSHTI JUJARE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Advanced', 'Web Development': 'Intermediate', 'Cloud Computing': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>['Google Data Analytics']</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>1.3</v>
+          <t>2023-present</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Third-year AI and Data Science student with front-end experience, interested in creating smart, user-friendly websites and AI-based applications.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from VISHWAKARMA UNIVERSITY, PUNE ( - )</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Winter Internship at CONSTROMAN AI (January 2025-Winter Internship) - Front End Development, Designing Marketing Booklets and Pamphlets</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GauravAmolGuddeti_CSE-AIML_ - Gaurav Guddeti.pdf</t>
+          <t>sau resume - Sayali Deore.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development', 'Cloud Computing']</t>
+          <t>Sayali Girdhar Deore</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced', 'Cloud Computing': 'Beginner'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.95</v>
+          <t>2023-current</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Motivated and hardworking student seeking to apply knowledge of data science and artificial intelligence in a real-world environment.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Hackathons, Research &amp; Presentations</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Python, Java, C Language</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Problem Solving, Communication, Teamwork, Fast Learner</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HTML, CSS, SQL, Excel, Power BI, Prompt Engineering</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>UG - B.TECH from Vishwakarma University, Pune ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Roomie link () - User-friendly web platform for finding compatible roommates and rental rooms.; Startup Research paper (Ongoing) - In-depth research project on startup ecosystems in India.; Sign language () - System to recognize and translate sign language gestures.; Sleep Effect on Maternal Health Research paper (Ongoing) - Research on impact of sleep patterns on maternal health.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Internship Student at Internpro, Pune, IN (June 2025 - July 2025 (Ongoing)) - Executed data cleaning and tokenization for sentiment analysis datasets, collaborated within a team</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shivam_Laxmikant_Deshmukh_AI&amp;DS_Resume - Shivam Laxmikant Deshmukh.pdf</t>
+          <t>VarunInamdar_ArtificialIntelligence - Varun Inamdar.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Cloud Computing']</t>
+          <t>VARUN NIKHIL INAMDAR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Advanced', 'Cloud Computing': 'Beginner'}</t>
+          <t>B.Tech AI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.75</v>
+          <t>07/2023 - 06/2027</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Motivated and detail-oriented AI and cybersecurity enthusiast currently pursuing B.Tech in CSE (AI). Adept at building AI-powered systems, real-time applications, and research-oriented solutions. Experienced in deploying AI models and integrating deep learning with web technologies. Passionate about</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Python, SQL, Flask, Go, Java, PyTorch, TensorFlow, Keras, Scikit-Learn, Pandas, OpenCV</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Leadership, Seeker Mindset, Team-player, Public Speaking, Problem-Solving, Creative, Quick learner</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Parallel Programming, Task Scheduling, Distributed Systems, Operating Systems, GCP</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>UG - B.Tech in Artificial Intelligence from Vishwakarma University, Pune, India (8.7 - 2027)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Smart Guard Surveillance System (Jan 2025 – April 2025) - Designed a smart surveillance system for fire, helmet, crowd, and weapon detection using deep learni; Cybersecurity AI Tutor and Evaluator (Jan 2025 - Present) - Developed a cybersecurity AI tutor using Ollama that delivers topic-wise explanations, adaptive MCQs; Resume Ranker AI (Apr 2025- May 2025) - Implemented a machine learning pipeline to extract and match keywords from resumes against job descr</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Business Intelligence Foundations with SQL, ETL and Data Warehousing Specialization by IBM (May 2025); Data Analytics Certificate by Google (June 2025)</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>at Drone Project Internship () - ...</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ShubhMali_AI&amp;DS - Shubh Mali.pdf</t>
+          <t>(JeremiahIsaac_Artificial Intelligence &amp; Data Science.pdf) - Jeremiah Isaac.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Jeremiah Isaac</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced'}</t>
+          <t>Bachelor of Technology</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.7</v>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Seeking a challenging internship opportunity in the field of Artificial Intelligence &amp; Data Science to apply and enhance technical skills and knowledge.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Volunteer in every cultural activities in my University, in different fields of Music, Sports, organization, Decor, and obtaining certificates for the mentioned and event management.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Certificate achieved for 'World Water Day' 'Ai Day'....</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BhoomiDhoka_ComputerScience_AI_DS - Bhoomi Dhoka.pdf</t>
+          <t>AnshulPatil_ArtificialIntelligence - Anshul Patil.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>['Web Development']</t>
+          <t>ANSHUL PATIL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.65</v>
-      </c>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>B.Tech student in AI &amp; ML seeking an opportunity to apply machine learning and data analysis skills to real-world projects. Eager to learn, contribute to innovative solutions, and grow in a dynamic tech environment.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Swimming, Cricket...</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Python (Backend Development), C Language, C++</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune (Not specified - Not specified); HSC - All India Senior School Certificate Examination (AISSCE) from Indian Language School, Lagos (Not specified - Not specified); SSC - All India Secondary School Examination (AISSE) from Not specified (Not specified - Not specified)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Mastering Basecamp for Project Management by LinkedIn Learning (Not specified); Energy Literacy Training by Energy Swaraj Foundation (Not specified); Nature-based Solutions for Disaster and Climate Resilience by UN (Not specified)</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rohitthakur_ai&amp;ml - Rohit Thakur.pdf</t>
+          <t>ShubhMali_AI&amp;DS - Shubh Mali.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Shubh Dinesh Mali</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0.55</v>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Third-year B.Tech student specializing in Artificial Intelligence and Data Science, with proficiency in C, C++, Python, data analysis, and full-stack development. Experienced in problem-solving, web and app development, and collaborative technical projects. Demonstrates strong leadership and teamwor</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University (55.33 - 2023); HSC -  from Rosary Junior College (68.80 - 2021); SSC -  from Sardar Dastur Hormazdiar High School ( - Expected 2027)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Real-Time Indian Sign Language Detection System () - Developed a real-time two-way communication system that detects and interprets Indian Sign Language ; Classroom Companion Website () - Created a centralized academic website using Wix for classmates, featuring timetables, notes, assign; Secure Online Voting System () - Developed a secure web-based voting platform ensuring authentication, data integrity, and transparen</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SaniyaShaikh_DataScience.pdf - Saniya Shaikh.pdf</t>
+          <t>GauravAmolGuddeti_CSE-AIML_ - Gaurav Guddeti.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Gaurav Amol Guddeti</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>BTech</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0.5</v>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Computer Science (AI &amp; ML)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Passionate about transforming data into intelligent solutions. I aim to innovate with AI and contribute to impactful projects while growing in a fast-paced, tech-driven environment.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Extra-curricular activities</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>UG - BTech from Vishwakarma University (8.15 - 2027); HSC - HSC from Vishwakarma College of Arts, Commerce and Science (70% - 2023); SSC - SSC from Sardar Dastur Hormazdiar High School (70% - 2021)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SmartJeb – AI-powered Expense Tracker () - A modern, secure financial companion that tracks expenses using AI-powered insights. Includes robust; Crop Disease Analyzer – AI for Agriculture () - Helps farmers detect crop diseases using AI-based image analysis.; Deblurryfy – Image Deblurring Tool () - Restores blurred images using Richardson-Lucy Deconvolution. Built using Streamlit.; Smart Traffic Signal System () - Adjusts signal timings dynamically based on real-time vehicle analysis using YOLOv8.; Jarvis ai () - A sophisticated AI-powered automation and chatbot system designed to assist with various tasks inclu</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>The Complete Python Bootcamp: From Zero to Hero by Udemy (2023); Generative AI Fundamentals by Google (2023); AI For India 2.0 by GUVI (2023); Review Paper Webinar Participation by Research Graduate (2023)</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AyushreeJadhav AI&amp;DS (1) - Ayushree Jadhav.pdf</t>
+          <t>SaniyaShaikh_DataScience.pdf - Saniya Shaikh.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development', 'Cloud Computing']</t>
+          <t>SANIYA SHAIKH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner', 'Web Development': 'Beginner', 'Cloud Computing': 'Beginner'}</t>
+          <t>BTech</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>0.5</v>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Aspiring Data Scientist with strong analytical skills. Currently pursuing BTech in Artificial Intelligence and Data Science (3rd Year) with hands-on experience in Python, SQL, Machine Learning, Data Visualization, and backend development using JDBC. Demonstrated ability to work on projects involving</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>UG - BTech from VISHWAKARMA UNIVERSITY, PUNE (8.1 - 2025); HSC - Senior Secondary from HHCP JR. COLLEGE, PUNE (72% - 2027); SSC - Secondary from DSK SCHOOL (ICSE BOARD) (90% - 2023)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Rescue Shield: AI-Powered Disaster Management System (March 2025) - Developed a disaster management software covering floods, earthquakes, and wildfires using React.js,; Energy Consumption Optimization using Smart Grid and IOT device -DSS project (Jan 2025 - April 2025) - Developed an energy consumption optimization system using smart grids and IoT data with data cleanin; Hotel Reservation System-JDBC project (Feb 2025 - April 2025) - Developed a Hotel Reservation System using JDBC with CRUD operations for room bookings, database int</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Data Science Intern at  (3rd Year) -</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rohit_Thakur_AI&amp;ML - Rohit Thakur.pdf</t>
+          <t>Rohitthakur_ai&amp;ml - Rohit Thakur.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Rohit Thakur</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>0.5</v>
+          <t>Year of Graduation: [Add Graduation Year]</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>To obtain a challenging position in a reputed organization where I can apply my skills in web development, embedded systems, and AI/ML to contribute to innovative projects and gain hands-on experience that furthers my professional growth.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Strong logical ...</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Web Development, Embedded Systems, AI/ML, Drones</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>C, C++, Java, JavaScript, Python, HTML, CSS, Git, VS Code, Eclipse</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University (7.9 / 10 - [Add Graduation Year])</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>DRDO Defence Drone () - Developed a drone prototype for defense surveillance and threat detection. Integrated camera modules; Shoplifting Detection System () - Designed a system using motion sensors and camera feeds to detect suspicious behavior. Alerts store</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>HTML and CSS for Web Designers: From Basics to Beautiful by Udemy · Instructor: Mehmood Khalil (June 20, 2025); Bring AI to Work Workshop by Google Workspace (June 4, 2025); Technology Job Simulation Certificate by Deloitte (via Forage) (June 2025)</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Technology Job Simulation Intern at Deloitte (via Forage Virtual Internship Program) (June 2025) - Completed hands-on tasks in coding and development. Gained insights into real-world project workflow</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SohamPatil_BTechAI&amp;DS - Soham Patil.pdf</t>
+          <t>MrudulaShinde - Mrudula Shinde.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Mrudula Shinde</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>['Google Data Analytics']</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>0.5</v>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Aspiring Data Analyst and B.Tech AI &amp; Data Science student eager to apply data analysis, visualization, and statistical skills in real-world projects. Passionate about uncovering actionable insights to support data-driven decisions.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Second Prize – 'Can You Case It?' Case Study Competition. Participated in workshops on Data Science, Power BI, SQL &amp; Statistics...</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Data Analysis, EDA, Data Cleaning, Visualization, Communication, ML (Basic)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SQL, Python, R, Java (Basic), PostgreSQL, Looker Studio, Power BI, Excel</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune (8.13/10 - 2027)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Rescue Shield – AI Powered Disaster Management System (Feb 2025 – Apr 2025) - Developed disaster software using React.js, Flask &amp; MySQL. Integrated real-time alerts, dynamic heat; Visualizing Market Trends: A Data-Driven Stock Market Dashboard for Investors (May 2025) - Created a dashboard to visualize 2024–2025 market trends using KPIs and charts for metrics like vola</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Tata Data Visualisation by Forage (July 2025); Deloitte Job Simulation by Forage (July 2025)</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Data Analyst Associate Intern at Excelerate (Virtual) (May 2025 – June 2025) - - Built interactive dashboards in Looker Studio to visualize KPIs. Performed EDA, cleaned data for s</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SumeetGupta_ArtificialIntelligence - Sumeet Shankar Gupta.pdf</t>
+          <t>DhruvGupta_ComputerEngineering_BtechAIandDS - Dhruv Gupta.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>DHRUV GUPTA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>0.45</v>
+          <t>2024-present</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>AI and DS</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Junior Teacher at Toppers Student Academy, Part-Time Sales Executive at Tilak Spares, Creative Intern at The Brand Mill</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>I have taken part in school debate and dance competitions</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Playing new video games, going to the gym, playing cricket occasionally, travelling</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Good conversationist, Quick learner, Good listener, Basics of Wix studio, Basics of SMM</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune ( - 2024-present)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Junior Teacher at Toppers Student Academy (TSA) (in 2023) - ; Part-Time Sales Executive at Tilak Spares (2024-May 2025) - ; Creative Intern at The Brand Mill (June 2025-) -</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VedantPandhare_Artificialintelligence - Vedant Pandhare.pdf</t>
+          <t>VishalShukla_CSE(AI&amp;ML) - Vishal Shukla.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning']</t>
+          <t>VISHAL SHUKLA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner'}</t>
+          <t>Bachelor of Technology in Computer Science Engineering</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Aug2023 - Aug2027</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AI &amp; ML</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Third-year BTech (AI &amp; ML) student with hands-on experience in Java, Spring Boot, and full-stack web development. Seeking a Software Engineering or Java Developer Internship to apply and enhance my backend and machine learning skills in real-world projects.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Spring Boot, MySQL, Git</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University (8.01 - Aug2027)</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Gemini Chatbot (Java, Spring Boot, React.js) - GitHub; File Compressor Web App (Java, Spring Boot, React.js) - GitHub Web app to upload, compress, decompress files using efficient algorithms. Created responsive ; Face Mask Detection (Python, CNN) - GitHub Built a CNN-based classifier to detect whether a person is wearing a mask or not. Trained on ; IMDB Sentiment Analysis (Python, NLP, Logistic Regression) - GitHub Analyzed 4500+ movie reviews to classify sentiment as positive/negative. Applied text preproc</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Java-hackerrank-certification by Maharashtra, Pune (+91-9284716995)</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kartik Gore - KARTIK GORE.pdf</t>
+          <t>AadityaDhanwate_Artificial Intelligence &amp; Data Science - Aaditya Dhanwate.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning']</t>
+          <t>Aaditya Dhanwate</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Beginner'}</t>
+          <t>BACHELOR OF TECHNOLOGY</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>0.4</v>
+          <t>2023 - 2027</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>AI &amp; Data Science undergraduate aiming to build a career as a Data Analyst. Strong interest in data interpretation, visualization, and statistical analysis. Looking for an opportunity to apply my knowledge in real-world projects and grow in a data-driven environment.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>National Science Day: Volunteered for science exhibitions (1st Year), Poster Competition: 1st Prize for creative design, Navachar C2P2 :Innovation Innovation Prototype based Project, Robotics: Built 4</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Python, SQL, R, C/C++</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Pandas, NumPy, Excel</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>UG - BACHELOR OF TECHNOLOGY from Vishwakarma University Pune ( - )</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>INSURANCE FRAUD DETECTION DASHBOARD USING POWER BI () - Built an interactive dashboard to detect fraud in insurance claims. Analyzed trends using demographi; SALES IMPROVEMENT ANALYSIS USING HYPOTHESIS TESTING () - Used T-tests, ANOVA, and Tukey HSD to evaluate the impact of a business intervention. Built and vali</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Certificate Folder Link by  ()</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>at  () -</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VishalShukla_CSE(AI&amp;ML) - Vishal Shukla(1).pdf</t>
+          <t>VedantPandhare_Artificialintelligence - Vedant Pandhare.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Vedant Pandhare</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Beginner', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>0.4</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>AI enthusiast passionate about solving real-world problems using advanced AI/ML frameworks and IoT technologies, with a proven track record of delivering innovative solutions and leading impactful initiatives.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma university ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Hand Gesture Detection for Alert Systems () - Designed an advanced model to recognize hand gestures for use in alert systems, improving human-mach; Time Series Forecasting for Crop Yield () - Optimized a forecasting model leveraging historical time series data to accurately predict crop yiel; Anomaly Detection () - Developed a robust real-time Anomaly detection system using popular frameworks like OpenCV and Tenso; Frame Interpolation on Raspberry Pi with Hailo-8L () - Designed the system to process incoming video feed on-the-fly, ensuring live interpolation without l; Document Summarizer (NLP Project) () - Built an NLP-based web application that automatically summarizes long and complex legal documents, e; Raspberry Pi-Based Applications () - Conceptualized, designed, and deployed innovative IoT solutions that utilized Raspberry Pi and edge ; AI-Powered Industrial Drones () - Spearheaded the development of AI-driven industrial drones. These drones utilized real-time AI capab</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Prathamesh_Pitale_AI - Prathamesh Pitale.pdf</t>
+          <t>AyushreeJadhav AI&amp;DS (1) - Ayushree Jadhav.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning']</t>
+          <t>Ayushree Jadhav</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Machine Learning': 'Intermediate'}</t>
+          <t>BTech</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>0.4</v>
+          <t>2020-2023</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Artificial intelligence and Data science</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Motivated and enthusiastic BTech student in Artificial Intelligence and Data Science with a strong interest in programming, data analysis, and modern technologies. Eager to learn, grow, and gain practical experience in the tech industry.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>UG - BTech from Vishwakarma university, pune ( - ); Diploma - Diploma In Computer Engineering from Guru Gobind Singh Polytechnic, Nashik ( - )</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>College Connect With Industry 4.0 Revolution Android App () - Built an Android application to link college students with industry trends and opportunities. Develo</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Project management by LinkedIn learning by  (); Certified with blue prism foundation training certificate by  (); Builders online series by AWS by  (); Certified with mobile application development course by  (); Python for beginners:Data Structure by coursera learner by  ()</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Web Development &amp; PHP Programming at Ayam Interactive () - Gained practical experience in web development. Learned PHP, frontend design, and backend integratio</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GautamSingh_AIDS-1 - Dipendra Thakur Hajam.pdf</t>
+          <t>ShaheedSofiPatel_Artificial Intelligence &amp; Data Science - Shaheed Patel.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development', 'Cloud Computing']</t>
+          <t>Shaheed Sofi Patel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Web Development': 'Intermediate', 'Cloud Computing': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>0.4</v>
-      </c>
+          <t>2023 - Present</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Motivated and detail-oriented undergraduate student pursuing a degree in Artificial Intelligence and Data Science, seeking an opportunity to apply technical skills and analytical knowledge in real-world projects.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University, Pune, Maharashtra (8.3 (up to current semester) - Present); HSC - Higher Secondary Certificate from PA University - MCES, Pune, Maharashtra (67.17% - 2023); SSC - Secondary School Certificate from FEHS, Thane, Maharashtra (77.80% - 2021)</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>System to efficiently generate and manage class schedules () - Minimizing conflicts and improving time allocation; Automated attendance tracking system () - Recording, managing, and reporting student attendance efficiently; Console-based application to manage employee records () - Functionalities for adding, updating, and retrieving employee data</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sufia Sayyed_AI - Sufia Sayyed.pdf</t>
+          <t>Rohit_Thakur_AI&amp;ML - Rohit Thakur.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Rohit Thakur</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>0.35</v>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>To obtain a challenging position in a reputed organization where I can apply my skills in web development, embedded systems, and AI/ML to contribute to innovative projects and gain hands-on experience that furthers my professional growth.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Strong logical thinking and problem-solving abilities. Quick learner and a good team player. Actively engaged in real-time embedded projects and tech innovations...</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>web development, embedded systems, AI/ML</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>C, C++, Java, JavaScript, Python, HTML, CSS, Git, VS Code, Eclipse</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University (8.27 / 10 - 2027)</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Shoplifting Detection System () - Designed a system using motion sensors and camera feeds to detect suspicious behavior. Alerts store</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>HTML and CSS for Web Designers: From Basics to Beautiful by Udemy (June 20, 2025); Bring AI to Work Workshop by Google Workspace (June 4, 2025); Technology Job Simulation Certificate by Deloitte (via Forage) (June 2025)</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Technology Job Simulation Intern at Deloitte (June 2025) - Completed hands-on tasks in coding and development. Gained insights into real-world project workflow</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Prajal_Jain_Artificial_Intelligence - Prajal Jain.pdf</t>
+          <t>PriteshShukla_AIADS - Pritesh Shukla.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning']</t>
+          <t>Pritesh Shukla</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Advanced'}</t>
+          <t>BTech Artificial Intelligence and Data Science</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>0.35</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built a pipeline to scrape tweets from financial influencers using snscrape and analyze sentiment using the VADER model to predict stock movement (TSLA). Merged tweet sentiment with daily stock price data (yfinance) to generate buy/sell signals and backtested the strategy based on next-day returns. </t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>UG - BTech from VISWAKARMA UNIVERSITY PUNE ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>SmartWaste – IoT &amp; Data-Driven Trash Management System () - Built an IoT-based smart trash monitoring system that alerts and optimizes trash collection routes b</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Project Management by  (); Data Science Course by  ()</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MrudulaShinde - Mrudula Shinde.pdf</t>
+          <t>Sufia Sayyed_AI - Sufia Sayyed.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development', 'Cloud Computing']</t>
+          <t>Sufia Nasir Sayyed</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Beginner', 'Cloud Computing': 'Intermediate'}</t>
+          <t>B.Tech AI &amp; DS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>2023 - 2025</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Third-year AI and Data Science engineering student, proficient in coding- C, C++, Python, data analysis, app &amp; web development, and problem-solving. Demonstrates leadership abilities through active participation in team projects and roles, with a passion for innovation and technology. Eager to secur</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Volunteered in both cultural and science-related events within the university and department. Developed strong leadership and organizational skills while contributing to the successful execution of mu</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Sports- Basketball, Badminton, Interior Styling, Driving, Reading Novels, Travelling</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>SSC -  from Rosary High School &amp; Junior College (87 - 2021); HSC -  from Mount Carmel Junior College (74.33 - 2023); UG - B.Tech AI &amp; DS from Vishwakarma University ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Research Paper Presentation on Estimation of Charge State () - Published and presented a research paper on the estimation of charge state in the International Conf; IoT-based Smart Accident Alert System Project (Ongoing) - Currently working on and writing a research paper on the development of a smart accident alert syste; Intrusion Face Detection System using AI/ML (Ongoing) - Currently working on and writing a research paper on an AI and ML-based system designed for campus s; AI-powered Digital Classroom App for Rural Students () - Built a mobile “Digital Classroom” app for a hackathon, where I worked on the frontend design using</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Project Management Course Certification by LinkedIn Learning ()</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>VishalShukla_CSE(AI&amp;ML) - Vishal Shukla.pdf</t>
+          <t>Sumeet_Vikramsingh_Sangwan - Sumeet Sangwan.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Sumeet Vikramsingh Sangwan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>0.3</v>
-      </c>
+          <t>2023 - Present</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>A passionate and curious B.Tech student specializing in Artificial Intelligence and Machine Learning, with a deep interest in backend development, game development, and cybersecurity. I aim to leverage my technical skills, creativity, and determination to contribute meaningfully to innovative projec</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Athletics, Swimming, Kickboxing, Mimicry Artist, Acting</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune ( - Present); HSC - Higher Secondary Education from Maharashtra State Board ( - ); SSC - SSC from Maharashtra State Board ( - )</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>image-recognition-cnn () - ; fake-news-detector () -</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bug Bounty Bootcamp by BloggersCon Vision Pvt. Ltd. in collaboration with Vishwakarma University (); Mastering Basecamp for Project Management by LinkedIn Learning ()</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AbhijitKarjiResume - Abhijit Karji.pdf</t>
+          <t>Kartik Gore - KARTIK GORE.pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>KARTIK GORE</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Web Development': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>0.3</v>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Winner of the Capstone Project 2024 at Vishwakarma University. Winner of the HackRank competition at Vishwakarma University. Decent Rank in HackerRank. Second runner-up in TPL (state-level cricket tournament). Skilled in Python and collaborative efforts to implement IoT and ML projects focused on en</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Python, SQL, Data Science, Machine Learning, Power BI, Tableau, Data Visualization, AI-Based Applications, Data Analysis, IOT</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>HSC - Higher Secondary from Takshila School, Ahmednagar ( - 2016); UG - B.Tech from Vishwakarma University, Pune ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Project Intern - CWPRS, Pune (Jan 2024 - July 2024) - Developed an IoT-based system integrated with machine learning to detect and prevent illegal cutting</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>SQL Intermediate &amp; Advanced by HackerRank ()</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Project Intern at Central Water and Power Research Station (Jan 2024 - July 2024) - Skilled in Python and collaborative efforts to implement an IoT and ML project focused on environmen</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AnshulPatil_ArtificialIntelligence - Anshul Patil.pdf</t>
+          <t>VishalShukla_CSE(AI&amp;ML) - Vishal Shukla(1).pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>VISHAL SHUKLA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>Bachelor of Technology in Computer Science Engineering</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>0.25</v>
+          <t>Aug2023 - Aug2027</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>AI &amp; ML</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Third-year BTech (AI &amp; ML) student with hands-on experience in Java, Spring Boot, and full-stack web development. Seeking a Software Engineering or Java Developer Internship to apply and enhance my backend and machine learning skills in real-world projects.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Java, JavaScript</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Spring Boot, React.js, REST API</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University (8.01 - Aug2027)</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Gemini Chatbot () - Java, Spring Boot, React.js; File Compressor Web App () - Java, Spring Boot, React.js; Face Mask Detection () - Python, CNN; IMDB Sentiment Analysis () - Python, NLP, Logistic Regression</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Java-hackerrank-certification by Maharashtra, Pune ()</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>at  () -</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Srushti Jujare-Resume - Srushti Jujare.pdf</t>
+          <t>Sumeet resume - Sumeet Sangwan.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Sumeet Vikramsingh Sangwan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>0.2</v>
-      </c>
+          <t>2023 - Present</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>A passionate and curious B.Tech student specializing in Artificial Intelligence and Machine Learning, with a deep interest in backend development, game development, and cybersecurity. I aim to leverage my technical skills, creativity, and determination to contribute meaningfully to innovative projec</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Athletics, Swimming, Kickboxing, Mimicry Artist, Acting</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune ( - Present); HSC - Higher Secondary Education from PVP Sainik School, Loni ( - ); SSC - SSC from Sun Bright School, Pune ( - )</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>image-recognition-cnn () - ; fake-news-detector () -</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bug Bounty Bootcamp by BloggersCon Vision Pvt. Ltd. in collaboration with Vishwakarma University (); Mastering Basecamp for Project Management by LinkedIn Learning ()</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sau resume - Sayali Deore.pdf</t>
+          <t>SohamPatil_BTechAI&amp;DS - Soham Patil.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Soham Patil</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>Bachelor of Technology</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>0.2</v>
+          <t>2023-Present</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Artificial intelligence &amp; Data science</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Aspiring Data Scientist with a strong foundation in AI, Data Science, and programming. Eager to apply analytical and technical skills to real-world challenges, contributing to organizational growth and personal development.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Member of Student Council, Vishwakarma University – Media and Strategy (2023–Present). Organized and promoted various campus-wide tech and cultural events. Passionate about portrait photography, conte</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Python, JavaScript, Java</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>HTML, CSS, ReactJS</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University ( - Present); HSC - High school from Vishwakarma College of Arts, Commerce and Science ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Weather Forecasting Ai ChatBot () - Developed a JavaScript-based weather app using OpenWeatherMap API. Implemented real-time weather upd; AI Chatbot in JavaScript () - Designed a conversational bot for general-purpose Q&amp;A. Focused on natural interaction flow using dec</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Google Data Analytics Professional Certificate by Google (); Project Management by  ()</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Regional Bussiness Head at Harmoniq (August 2024 - September 2024) - Successfully led and managed event operations across Pune, collaborating with venue partners and ens</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sufiyanshahnawazansari.pdf - Sufiyan Ansari.pdf</t>
+          <t>AbhijitKarjiResume - Abhijit Karji.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Abhijit karji</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech Computer Science Engineering</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>0.2</v>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Machine Learning</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Highly skilled programmer with will to learn and improve. Efficient in Frontend Development. Possess strong problem-solving skills, ability to work in fast paced environment, and good communication skills.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Java, DBMS, Python</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Communication Skills, Quick Learner, Team Player</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>C/C++, Git, Javascript</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University ( - 2024)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>High Payload Drone (March 2024-Present) - Designed and deployed a high payload drone as part of a competition. Responsible for designing and i</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Hardware Team Lead at  () - Designed and integrated critical hardware systems for a high payload drone project.</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AadityaDhanwate_Artificial Intelligence &amp; Data Science - Aaditya Dhanwate.pdf</t>
+          <t>PriyantDharwarkar_ComputerEngineeringInAi&amp;Ds - Priyant Dharwarkar.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>['Python']</t>
+          <t>Priyant Y. Dharwarkar</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>{'Python': 'Advanced'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>0.2</v>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Computer Science in Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>To obtain a challenging position where I can utilize my strong foundation in programming, database management, and hands-on technical skills to contribute effectively to software development and problem-solving tasks.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>C Programming, C++, Core Java</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Advanced Java, Python, SQL</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University Pune ( - 2023-2024)</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Data Structures Project () - Developed a centralized system to automate the creation and management of academic timetables. Imple</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Diploma in - C Programming | C++ | Core Java | Advanced Java | Python | SQL | Data Structure by  ()</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>at  () -</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ShaheedSofiPatel_Artificial Intelligence &amp; Data Science - Shaheed Patel.pdf</t>
+          <t>AniketMane_B.TECH_CSE-AI - Aniket Mane.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Aniket Mane</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>Diploma</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>0.2</v>
+          <t>2020-2023</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Experienced HMI Graphics Engineer with demonstrated expertise in delivering high-quality, Human‑Machine Interface (HMI) solutions at Honeywell Automation India Limited (HAIL). Skilled in developing both static and dynamic HMI visuals, and providing independent on-site client support at CPCL Chennai </t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Diploma - Computer Engineering from Trinity Polytechnic ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>SunCore DSP-to-HMI conversion () - Migration graphics development project; KOC GC‑15 and GC‑23 unit graphics for Kuwait Oil Company () - Migration graphics development project; Java shape-template development for GPIC (Gulf Petrochemical Industries Company) () - Migration graphics development project</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>HMI Graphics Engineer at Honeywell (Randstad Payroll) (09/2023 – present) - Designed high-impact static graphics and advanced dynamic shape modifications, collaborated with cro</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sumeet_Vikramsingh_Sangwan - Sumeet Sangwan.pdf</t>
+          <t>Shivam_Laxmikant_Deshmukh_AI&amp;DS_Resume - Shivam Laxmikant Deshmukh.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Shivam Laxmikant Deshmukh</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>B-Tech</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>0.2</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Aspiring Data Analyst with a strong foundation in machine learning, data visualization, and real-time systems. Experienced in solving real-world problems using Python, SQL, and TensorFlow. Award-winning capstone project presenter with practical experience in open-source tool analysis and emergency c</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>UG - B-Tech from Vishwakarma University, Pune ( - 2027); HSC - Higher Secondary from Blue Blees College, Nanded ( - )</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Emergency Beacon – Real-time Image Recognition for Swift Assistance (Jan 2024 - July 2024) - Developed a real-time hand gesture recognition system using TensorFlow and OpenCV. Improved emergenc; Capstone Project – Comparative Study on FOSS Data Analysis Tools () - Analyzed and compared 5 open-source data analysis software. Published a research paper on findings. ; Advertising Dataset Analysis (Python + R) () - Tech Stack: Python (EDA), R (Z-scores, regression, boxplots, scatter plots). Goal: Predict the effec</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>SQL Intermediate &amp; Advanced by HackerRank (); Data Visualization by LinkedIn ()</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sumeet resume - Sumeet Sangwan.pdf</t>
+          <t>SrushtiNawghane_AIDS - Srushti Nawghane.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Srushti Gajanan Nawghane</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>0.2</v>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Aspiring Artificial Intelligence &amp; Data Science student with a passion for technology, data driven problem solving, and continuous learning. Seeking opportunities to apply and expand my skills through real-world projects, internships, or research. Passionate about building intelligent solutions that</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Research &amp; Presentations: Capstone Project – Air Monitoring Device, Volunteering &amp; Participation: Innovation Fest 2024-Participation, National Science Day – Volunteer and Designed and built a function</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>HSC - Graduated 12th from B.H Chate School&amp;Junior College Pune ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Air Monitoring Device () - Written Research paper</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Volunteering Certificate: National Science Day by  (); Volunteering Certificate: World Water Day by  (); Introduction to Artificial Intelligence: Infosys Springboard by  (2024)</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>RESEARCH EXPERIENCE- Capstone Project at  () - Topic: Air Monitoring Device</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Vrushali_nalawade_Resume[1] (1) - Vrushali Nalawade.pdf</t>
+          <t>Prathamesh_Pitale_AI - Prathamesh Pitale.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning', 'Web Development']</t>
+          <t>Prathamesh Pitale</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Machine Learning': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>Bachelor of Technology</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>0.2</v>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motivated and detail-oriented third-year undergraduate student in Artificial Intelligence and Data Science seeking opportunities to apply technical knowledge, analytical skills, and a passion for innovation in real-world projects and internships. Eager to contribute to impactful AI-driven solutions </t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University, Pune ( - 2027); HSC -  from Vishwakarma College of Arts, Commerce and Science ( - 2023)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Google Project Management by Coursera (); AI for Everyone by Coursera (); Data Science Specialization by  (); Project Management by  (); Energy Literacy Training [EVS] by  ()</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>JUSTY RESUME - Bardeskar John.pdf</t>
+          <t>Shrutigapat_AIDS.PDF - Shruti Gapat.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Shruti Gapat</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Web Development': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>0.2</v>
+          <t>2023 - current</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Aspiring Artificial Intelligence &amp; Data Science student with a passion for technology, data-driven problem solving, and continuous learning. Seeking opportunities to apply and expand my skills through real-world projects, internships, or research. Passionate about building intelligent solutions that</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>HSC - 12th from CHATE COLLEGE, PUNE ( - 2023); UG - B.Tech from Vishwakarma University, Pune ( - current)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Smart Traffic Light System Using AI (Ongoing) - Designing a traffic control simulation that detects ambulances in real-time via object detection and; Air Monitoring Device () - Wrote Research paper</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Volunteering Certificate: National Science Day by  (); Volunteering Certificate: World Water Day by  (); Introduction to Natural Language Processing by Infosys Springboard (2024); Introduction to Data Science by Infosys Springboard (2024); Introduction to Artificial Intelligence by Infosys Springboard (2024); Generative AI Unleashing by Infosys Springboard (2024); Introduction to Deep Learning by Infosys Springboard (2024); Time Management by Infosys Springboard (2024); Computer vision by Infosys Springboard (2024)</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>RESEARCH EXPERIENCE- Capstone Project at  () - Topic: Air Monitoring Device, Wrote Research paper</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Resume - Himanshu Sankhla.pdf</t>
+          <t>Vrushali_nalawade_Resume[1] (1) - Vrushali Nalawade.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Vrushali Mahesh Nalawade</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>0.2</v>
+          <t>2023-current</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Aspiring Data Science professional with a strong interest in Machine Learning. Actively learning ML to build a strong foundation in the field.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Hackathons, Research &amp; Presentations, Volunteering &amp; Participation</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Programming: Python, Java, C Language, Web Technologies: HTML, CSS, Data Tools: SQL, Excel, Power BI, Other Tools: Prompt Engineering, Video Editing, Soft Skills: Problem Solving, Communication, Teamwork, Adaptability, Fast Learner, Note-taking</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>UG - B TECH from Vishwakarma University, Pune ( - )</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Home Security System using Computer Vision () - Developed a basic surveillance system using traditional computer vision techniques to detect motion</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Volunteering Certificate - National Science Day by  (); Volunteering Certificate - World Water Day by  (); Certificate - VU-BU Hackathon (Consolation Prize) by  (); Certificate - Vyoma Hackathon (Participant) by  ()</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Internship Student at Internpro, Pune, IN (June 2025 - July 2025 (Ongoing)) - Executed data cleaning and tokenization for sentiment analysis datasets. Collaborated within a team</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AarohDharmadhikari_AIDS - Aaroh Dharmadhikari.pdf</t>
+          <t>Prajal_Jain_Artificial_Intelligence - Prajal Jain.pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>['Python', 'Machine Learning']</t>
+          <t>Prajal Jain</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Machine Learning': 'Beginner'}</t>
+          <t>Bachelor's in Technology</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>0.15</v>
-      </c>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Mechatronics</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Experienced in Mechatronics, Robotics, AI, and Machine Learning with strong skills in Python, C++, MATLAB, and various design &amp; simulation tools.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Mechatronics &amp; Robotics, AI &amp; Machine Learning, Programming Languages</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Analytical Thinking, Problem Solving, Team Collaboration</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Python, C++, MATLAB</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>UG - Bachelor's in Technology from Vishwakarma University, Pune, India (7.9 - 2027); Diploma - Diploma in Mechatronics from Indo German Tool Room, Aurangabad, India (7.9 - 2024)</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Video Classifier Recycle Bin (Jan 2024 - May 2024) - Developed an AI-based video classification system to sort biomedical waste from live footage. Achiev; Arduino-Powered Drone (Jul 2022 - Nov 2022) - Designed and assembled a custom quadcopter using Arduino and IMU sensors. Enhanced reliability with ; AI Cyber Coach (Jan 2025 - May 2025) - Built an AI-powered learning assistant with a chatbot for solving student queries. Enabled mentor da</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Neural Networks and Deep Learning by  (2027); Improving Deep Neural Networks by  (2027); AI For Everyone by  (2027); Structuring Machine Learning Projects by  (2027); SQL for Data Science by  (2027); Linux &amp; Shell Scripting by  (2027)</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PriyantDharwarkar_ComputerEngineeringInAi&amp;Ds - Priyant Dharwarkar.pdf</t>
+          <t>GautamSingh_AIDS-1 - Dipendra Thakur Hajam.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>GAUTAM SINGH</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Web Development': 'Beginner'}</t>
+          <t>Bachelor of Technology</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>0.15</v>
-      </c>
+          <t>2024-2027</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Detail-oriented and motivated computer engineering student with a strong foundation in programming, data structures, and system design. Skilled in translating theoretical concepts into real-world applications, particularly in software development, AI, and embedded systems. Eager to contribute techni</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from VISHWAKARMA University ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Developing a smart facial recognition system enhanced with Natural Language Processing NLP (ONGOING) - To interpret verbal commands and provide interactive responses. Integrating OpenCV for face detectio</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Social Network by https://forage-uploads-prod.s3.amazonaws.com/completion-certificates/9PBTqmSxAf6zZTseP/io9DzWKe3PTsiS6GG_9PBTqmSxAf6zZTseP_ZJW54tBeXPy2TMY4x_1751515955017_completion_certificate.pdf (); Social Network by https://forage-uploads-prod.s3.amazonaws.com/completion-certificates/9PBTqmSxAf6zZTseP/udmxiyHeqYQLkTPvf_9PBTqmSxAf6zZTseP_ZJW54tBeXPy2TMY4x_1751430696288_completion_certificate.pdf ()</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SrushtiNawghane_AIDS - Srushti Nawghane.pdf</t>
+          <t>ParjanyaKandala_CSEAI - Parjanya Phanikumar Kandala.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Parjanya Kandala</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>0.15</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>To gain practical experience and enhance my skills by contributing to real world projects and learning through internship opportunities.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>C, Java, Python</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>HTML, MySQL</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma Univeristy, Pune (NA - 2027)</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Obstacle Avoiding Car using Arduino (NA) - Developed an obstacle-detection vehicle using Arduino and ultrasonic sensors as part of a collaborat</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>BI Foundations with SQL, ETL and Data Warehousing by COURSERA (NA); ETL and Data Pipelines with Shell, Airflow and Kafka by IBM (NA); Databases and SQL for Data Science with Python by COURSERA (NA); Data Warehouse Fundamentals by COURSERA (NA); BI Dashboards with IBM Cognos Analytics and Google Looker by COURSERA (NA); Hands-on Introduction to Linux Commands and Shell Scripting by COURSERA (NA)</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Shrutigapat_AIDS.PDF - Shruti Gapat.pdf</t>
+          <t>NihalPardeshi_ComputerEngineeringAIML - Nihal Pardeshi.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>NIHAL PARDESHI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>0.15</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CSE (AI/ML Specialization)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>AI/ML undergrad with hands-on exposure to core machine learning concepts including regression, classification, and clustering. Built multiple proof-of-concept projects involving sentiment analysis and mood detection using Hugging Face models and cloud tools like AWS. Comfortable with Python, Pandas,</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Hackathon Moderator: Organized and managed a successful college hackathon, fostering collaboration among participants.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune ( - 2027)</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Moodify (Under Development) - Affective Computing Music Recommendation System (May. 2024 – Present) - Developed a web application that detects user's mood through emoji slider and text input to recommen; 100 Days of ML (Nov. 2024 – Present) - Public initiative simplifying ML workflows and concepts for beginners. Published insights on feature; Anxiety Detection Tool (Oct. 2024) - Developed an offline anxiety detection tool using Hugging Face's DistilBERT for real-time sentiment ; Pune Waste Classification (Toy ML Project) (Sep. 2024) - Cleaned Pune waste dataset using Pandas; visualized data with Matplotlib.</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ParjanyaKandala_CSEAI - Parjanya Phanikumar Kandala.pdf</t>
+          <t>BhoomiDhoka_ComputerScience_AI_DS - Bhoomi Dhoka.pdf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>BHOOMI DHOKA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate', 'Web Development': 'Beginner'}</t>
+          <t>Bachelor of Technology</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>0.15</v>
-      </c>
+          <t>Aug 2023 - June 2027</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence and Data Science</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Frontend developer and AI student focused on building fast, responsive React applications and exploring data analysis to inform better UX decisions. Seeking an internship to apply performance auditing, modular UI design, and real-world data skills.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Participated in Can You Case It?, a university-level case competition applying teamwork and problem-solving to real-world business scenarios.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Maintain active, well-documented frontend projects on GitHub, using version control and clear commit practices.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Responsive Web Design, API Integration, User Input &amp; Form Handling</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Teamwork &amp; Collaboration, Problem Solving, Effective Communication</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>React.js, JavaScript (ES6+), HTML</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>UG - Bachelor of Technology from Vishwakarma University ( - June 2027)</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>RecipeRipple | Web-Based Recipe Discovery App () - Designed a mobile-first UI scoring 90+ Lighthouse Performance and 0 CLS across Chrome, Firefox, and ; Task Navigator Pro | Personal Task Management App () - Built a responsive task manager scoring ~90 in performance with zero total blocking time. Developed</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>(JeremiahIsaac_Artificial Intelligence &amp; Data Science.pdf) - Jeremiah Isaac.pdf</t>
+          <t>SumeetGupta_ArtificialIntelligence - Sumeet Shankar Gupta.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>['Python', 'Web Development']</t>
+          <t>Sumeet Shankar Gupta</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{'Python': 'Beginner', 'Web Development': 'Beginner'}</t>
+          <t>B.Tech in AI &amp; DS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>0.1</v>
-      </c>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Data Science</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Dedicated and detail-oriented AI &amp; Data Science undergraduate with a passion for building smart solutions and solving real-world problems. Seeking opportunities to apply technical knowledge in software development, data analytics, and intelligent systems through hands-on industry projects.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>UG - B.Tech in AI &amp; DS from Vishwakarma University (8.46 - 2027); HSC - Class XII (Science) from Swami Vivekanand Kanistha Mahavidyalaya, Mumbai (70% - 2023); SSC - Class X from Model High School, Mumbai (81.40% - 2021)</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Alumni Management System () - GUI-based alumni portal using hash tables and linked lists.; E-commerce Sales Forecasting () - Sales prediction via time-series and regression models.; Print Job Scheduler () - Print scheduler with FIFO/Priority mode and GUI.; Real Estate Management System () - Property and client management with file I/O and trees.; Car Rental System () - Terminal-based rental system with car availability tracking.; Free Analytics Software System – Capstone Project () - Won 1st Prize in Capstone 2024 for creating a no-cost analytics system for real-time data tracking.</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>SQL (Advanced) by HackerRank (Apr 2025); SQL (Intermediate) by HackerRank (Feb 2025); SQL (Basic) by HackerRank (Feb 2025); Certified Associate in Project Management (CAPM)® Tips by LinkedIn Learning (Mar 2025); Generative AI Powered Project Plans by LinkedIn Learning (Mar 2025); Project Management Foundations by LinkedIn Learning (Jan 2025)</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PriteshShukla_AIADS - Pritesh Shukla.pdf</t>
+          <t>Resume - Himanshu Sankhla.pdf</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>['Python']</t>
+          <t>Himanshu Sankhla</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{'Python': 'Intermediate'}</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>MansiBharatEvre_ComputerEngineering - Mansi Evre.pdf</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>['Machine Learning']</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>{'Machine Learning': 'Beginner'}</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>AniketMane_B.TECH_CSE-AI - Aniket Mane.pdf</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>['Python']</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>{'Python': 'Beginner'}</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>DhruvGupta_ComputerEngineering_BtechAIandDS - Dhruv Gupta.pdf</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CSE (AI&amp;ML)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>App Developer, Game Developer, AI &amp; ML engineer</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>App Development (Android Native), Python, Java</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>UG - B.Tech from Vishwakarma University, Pune (8.54 - 2025); XII - CBSE from Central Academy Sr. Sec. School (73% - 2023)</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Unit Converter () - A simple Jetpack Compose unit conversion app for length measurements. Users enter a value, select in; Shopping List () - The app allows users to add, edit, and delete shopping items dynamically. It features a clean and re</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>